<commit_message>
puzzles: clarify arithmetic balance queries
</commit_message>
<xml_diff>
--- a/task-reviews/puzzles/task_puzzles_arithmetic_balance_value/task_puzzles_arithmetic_balance_value.xlsx
+++ b/task-reviews/puzzles/task_puzzles_arithmetic_balance_value/task_puzzles_arithmetic_balance_value.xlsx
@@ -4285,17 +4285,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4304,12 +4304,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 11}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 11}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -4349,17 +4349,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4368,12 +4368,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -4413,17 +4413,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number belongs to the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What integer belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number belongs to the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What integer belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4432,12 +4432,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -4477,17 +4477,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Which integer matches the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Which number completes the final query row?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Which integer matches the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Which number completes the final query row?
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4496,12 +4496,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -4541,17 +4541,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Which integer matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Which number completes the final query row?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Which integer matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Which number completes the final query row?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4560,12 +4560,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 11}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 11}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -4605,17 +4605,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4624,12 +4624,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 3}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -4669,17 +4669,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4688,12 +4688,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -4733,17 +4733,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4752,12 +4752,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -4797,17 +4797,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>You are given an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Which integer matches the highlighted query box?
+          <t>You are given an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Which number completes the final query row?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>You are given an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Which integer matches the highlighted query box?
+          <t>You are given an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Which number completes the final query row?
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4816,12 +4816,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -4861,17 +4861,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Determine the value represented by the highlighted query symbol.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Determine the value represented by the highlighted query symbol.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4880,12 +4880,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4925,17 +4925,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Which integer matches the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Which number completes the final query row?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Which integer matches the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Which number completes the final query row?
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -4944,12 +4944,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -4989,17 +4989,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Determine the value represented by the highlighted query symbol.
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Determine the value represented by the highlighted query symbol.
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5008,12 +5008,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -5053,17 +5053,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Which integer matches the highlighted query box?
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Which number completes the final query row?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Which integer matches the highlighted query box?
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Which number completes the final query row?
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5072,12 +5072,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 3}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -5117,17 +5117,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5136,12 +5136,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -5181,17 +5181,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5200,12 +5200,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 9}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -5245,17 +5245,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5264,12 +5264,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -5309,17 +5309,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Determine the value represented by the highlighted query symbol.
+          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Determine the value represented by the highlighted query symbol.
+          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5328,12 +5328,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -5373,17 +5373,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number belongs to the symbol in the highlighted query box?
+          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What integer belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number belongs to the symbol in the highlighted query box?
+          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What integer belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5392,12 +5392,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -5437,17 +5437,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What number belongs to the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What integer belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What number belongs to the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What integer belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5456,12 +5456,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -5501,17 +5501,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What number belongs to the symbol in the highlighted query box?
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What integer belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What number belongs to the symbol in the highlighted query box?
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What integer belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5520,12 +5520,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 11}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 11}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -5565,17 +5565,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Determine the value represented by the highlighted query symbol.
+          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Determine the value represented by the highlighted query symbol.
+          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5584,12 +5584,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -5629,17 +5629,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Which integer matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Which number completes the final query row?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Which integer matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Which number completes the final query row?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5648,12 +5648,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5693,17 +5693,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Determine the value represented by the highlighted query symbol.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Determine the value represented by the highlighted query symbol.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Determine the integer that belongs in the question-mark query box.
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5712,12 +5712,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -5757,17 +5757,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use the shown equalities to solve the highlighted query symbol.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use the shown equalities to solve the question-mark box.
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5776,12 +5776,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 9}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -5821,17 +5821,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":7}</t>
+{"evidence":[[574,508,686,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -5840,12 +5840,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5982,17 +5982,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>You are given an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>You are given an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>You are given an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>You are given an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6001,12 +6001,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 4}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -6046,17 +6046,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Use all three equality panels to determine the highlighted query value.
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Use all three equality panels to determine the highlighted query value.
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6065,12 +6065,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -6110,17 +6110,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Solve the full equality chain and report the highlighted query value.
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Solve the full equality chain and report the missing question-mark value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Solve the full equality chain and report the highlighted query value.
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Solve the full equality chain and report the missing question-mark value.
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6129,12 +6129,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 2}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -6174,17 +6174,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6193,12 +6193,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -6238,17 +6238,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6257,12 +6257,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 9}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -6302,17 +6302,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Solve the full equality chain and report the highlighted query value.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Solve the full equality chain and report the missing question-mark value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Solve the full equality chain and report the highlighted query value.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Solve the full equality chain and report the missing question-mark value.
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6321,12 +6321,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -6366,17 +6366,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What is the value of the symbol in the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What is the value of the symbol in the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 14}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -6430,17 +6430,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6449,12 +6449,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 6}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -6494,17 +6494,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6513,12 +6513,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 16}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 16}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -6558,17 +6558,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What number matches the highlighted query box?
+          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What number matches the highlighted query box?
+          <t>The image shows an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6577,12 +6577,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -6622,17 +6622,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6641,12 +6641,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 12}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -6686,17 +6686,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What number matches the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What number matches the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6705,12 +6705,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 14}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -6750,17 +6750,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Solve the full equality chain and report the highlighted query value.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Solve the full equality chain and report the missing question-mark value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Solve the full equality chain and report the highlighted query value.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Solve the full equality chain and report the missing question-mark value.
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6769,12 +6769,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 18}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 18}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -6814,17 +6814,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6833,12 +6833,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -6878,17 +6878,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6897,12 +6897,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -6942,17 +6942,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What number matches the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What number matches the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -6961,12 +6961,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 8}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -7006,17 +7006,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7025,12 +7025,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 9}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -7070,17 +7070,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Read the equality puzzle and determine the number that matches the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Read the equality puzzle and determine the number that completes the query row. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7089,12 +7089,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 2}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -7134,17 +7134,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Solve the full equality chain and report the highlighted query value.
+          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Solve the full equality chain and report the missing question-mark value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Solve the full equality chain and report the highlighted query value.
+          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Solve the full equality chain and report the missing question-mark value.
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7153,12 +7153,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -7198,17 +7198,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7217,12 +7217,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 5}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -7262,17 +7262,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Determine the integer represented by the highlighted query symbol.
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Determine the integer that completes the final query row.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Determine the integer represented by the highlighted query symbol.
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Determine the integer that completes the final query row.
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7281,12 +7281,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 12}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -7326,17 +7326,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number matches the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number matches the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7345,12 +7345,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 8}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -7390,17 +7390,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7409,12 +7409,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -7454,17 +7454,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>You are given an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>You are given an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>You are given an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use all three equality panels to determine the highlighted query value.
+          <t>You are given an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7473,12 +7473,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 5}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -7518,17 +7518,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Use all three equality panels to determine the highlighted query value.
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":5}</t>
+{"evidence":[[574,508,686,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Use all three equality panels to determine the highlighted query value.
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Use all three equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7537,12 +7537,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 524.0, 568.0, 636.0]], "answer": 20}</t>
+          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 20}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 524.0, 568.0, 636.0]]</t>
+          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -7679,17 +7679,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7698,12 +7698,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -7743,17 +7743,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>You are given a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7762,12 +7762,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 16}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 16}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7807,17 +7807,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Solve the equality chain and report the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Solve the equality chain and report the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7826,12 +7826,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 14}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -7871,17 +7871,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7890,12 +7890,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -7935,17 +7935,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What number matches the highlighted query box?
+          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What number matches the highlighted query box?
+          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -7954,12 +7954,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -7999,17 +7999,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>The image shows an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8018,12 +8018,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -8063,17 +8063,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Solve the equality chain and report the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Solve the equality chain and report the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8082,12 +8082,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 3}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -8127,17 +8127,17 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8146,12 +8146,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -8191,17 +8191,17 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number matches the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number matches the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8210,12 +8210,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -8255,17 +8255,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8274,12 +8274,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -8319,17 +8319,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8338,12 +8338,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -8383,17 +8383,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8402,12 +8402,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 18}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 18}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -8447,17 +8447,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What number matches the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number belongs in the question-mark query box?
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8466,12 +8466,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -8511,17 +8511,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Determine the integer represented by the highlighted query symbol.
+          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Determine the integer that completes the final query row.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Determine the integer represented by the highlighted query symbol.
+          <t>Look at the equality puzzle in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Determine the integer that completes the final query row.
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8530,12 +8530,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -8575,17 +8575,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Use the two equality panels to determine the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Use the two equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Use the two equality panels to determine the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Use the two equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8594,12 +8594,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 16}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 16}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -8639,17 +8639,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Determine the integer represented by the highlighted query symbol.
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Determine the integer that completes the final query row.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Determine the integer represented by the highlighted query symbol.
+          <t>The image shows a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Determine the integer that completes the final query row.
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8658,12 +8658,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -8703,17 +8703,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8722,12 +8722,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -8767,17 +8767,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use the two equality panels to determine the highlighted query value.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use the two equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Use the two equality panels to determine the highlighted query value.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Use the two equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8786,12 +8786,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -8831,17 +8831,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Solve the equality chain and report the highlighted query value.
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. Solve the equality chain and report the highlighted query value.
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with key "answer".
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8850,12 +8850,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -8895,17 +8895,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What is the value of the symbol in the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Work from the shown equalities to find the value of the highlighted symbol. What is the value of the symbol in the highlighted query box?
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Work from the shown equalities to find the number that fills the question-mark box. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8914,12 +8914,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -8959,17 +8959,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Solve the equality chain and report the highlighted query value.
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Solve the equality chain and report the highlighted query value.
+          <t>Look at the equality puzzle in the image: an outline-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -8978,12 +8978,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -9023,17 +9023,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Solve the equality chain and report the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Use the stacked equality panels in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Solve the equality puzzle and report the integer value of the highlighted query box. Solve the equality chain and report the highlighted query value.
+          <t>Use the stacked equality panels and query row in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Solve the equality puzzle and report the integer value that belongs in the question-mark query box. Solve the equality chain and report the missing question-mark value.
 Return a valid JSON object with key "answer".
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -9042,12 +9042,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -9087,17 +9087,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Determine the integer represented by the highlighted query symbol.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Determine the integer that completes the final query row.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. Determine the integer represented by the highlighted query symbol.
+          <t>Work from the equality-style arithmetic puzzle shown in the image: an arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. Determine the integer that completes the final query row.
 Return a valid JSON object with key "answer".
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -9106,12 +9106,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -9151,17 +9151,17 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Use the two equality panels to determine the highlighted query value.
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Use the two equality panels to determine the question-mark query value.
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Use the equality panels to determine the value of the highlighted query symbol. Use the two equality panels to determine the highlighted query value.
+          <t>Look at the equality puzzle in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Use the equality panels to determine what number replaces the question mark in the query row. Use the two equality panels to determine the question-mark query value.
 Return a valid JSON object with key "answer".
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -9170,12 +9170,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 14}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -9215,17 +9215,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number should replace the question mark?
 Return a valid JSON object with keys "evidence" and "answer" in that order.
-Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the highlighted query box.
+Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[456,508,568,620]],"answer":8}</t>
+{"evidence":[[574,508,686,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers separated by an explicit equals sign, plus one highlighted query box below the panels. Infer the value represented by the symbol in the highlighted query box. What is the value of the symbol in the highlighted query box?
+          <t>Work from the equality-style arithmetic puzzle shown in the image: a card-style arithmetic equality puzzle with stacked panels of boxed symbols and numbers, explicit plus and equals signs, and a final query row that ends with a question-mark box. Infer the missing number in the final query row. What number should replace the question mark?
 Return a valid JSON object with key "answer".
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
@@ -9234,12 +9234,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[456.0, 449.0, 568.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[456.0, 449.0, 568.0, 561.0]]</t>
+          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">

</xml_diff>

<commit_message>
puzzles: refine balance operator spacing
</commit_message>
<xml_diff>
--- a/task-reviews/puzzles/task_puzzles_arithmetic_balance_value/task_puzzles_arithmetic_balance_value.xlsx
+++ b/task-reviews/puzzles/task_puzzles_arithmetic_balance_value/task_puzzles_arithmetic_balance_value.xlsx
@@ -4290,7 +4290,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -4304,12 +4304,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 11}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 11}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -4354,7 +4354,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -4368,12 +4368,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -4418,7 +4418,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -4432,12 +4432,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -4482,7 +4482,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4496,12 +4496,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -4546,7 +4546,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4560,12 +4560,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 11}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 11}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -4610,7 +4610,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4624,12 +4624,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 3}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -4674,7 +4674,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -4688,12 +4688,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -4738,7 +4738,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4752,12 +4752,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -4802,7 +4802,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -4816,12 +4816,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -4866,7 +4866,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -4880,12 +4880,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4930,7 +4930,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -4944,12 +4944,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -4994,7 +4994,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -5008,12 +5008,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -5058,7 +5058,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -5072,12 +5072,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 3}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -5122,7 +5122,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -5136,12 +5136,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -5186,7 +5186,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -5200,12 +5200,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 9}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -5250,7 +5250,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -5264,12 +5264,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -5314,7 +5314,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -5328,12 +5328,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -5378,7 +5378,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -5392,12 +5392,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -5442,7 +5442,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -5456,12 +5456,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -5506,7 +5506,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -5520,12 +5520,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 11}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 11}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -5570,7 +5570,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -5584,12 +5584,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -5634,7 +5634,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -5648,12 +5648,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5698,7 +5698,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -5712,12 +5712,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -5762,7 +5762,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -5776,12 +5776,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 9}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -5826,7 +5826,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":7}</t>
+{"evidence":[[610,508,722,620]],"answer":7}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -5840,12 +5840,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5987,7 +5987,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -6001,12 +6001,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 4}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -6051,7 +6051,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -6065,12 +6065,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -6115,7 +6115,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -6129,12 +6129,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 2}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -6179,7 +6179,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -6243,7 +6243,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -6257,12 +6257,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 9}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -6307,7 +6307,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -6321,12 +6321,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -6371,7 +6371,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 14}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -6435,7 +6435,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -6449,12 +6449,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 6}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -6499,7 +6499,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -6513,12 +6513,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 16}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 16}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -6563,7 +6563,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -6577,12 +6577,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -6627,7 +6627,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -6641,12 +6641,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 12}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -6691,7 +6691,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -6705,12 +6705,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 14}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -6755,7 +6755,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -6769,12 +6769,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 18}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 18}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -6819,7 +6819,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -6833,12 +6833,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -6883,7 +6883,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -6897,12 +6897,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -6947,7 +6947,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -6961,12 +6961,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 8}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -7011,7 +7011,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -7025,12 +7025,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 9}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -7075,7 +7075,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -7089,12 +7089,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 2}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -7139,7 +7139,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -7153,12 +7153,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -7203,7 +7203,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -7217,12 +7217,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 5}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -7267,7 +7267,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -7281,12 +7281,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 12}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -7331,7 +7331,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -7345,12 +7345,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 8}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -7395,7 +7395,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -7409,12 +7409,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -7459,7 +7459,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -7473,12 +7473,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 5}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -7523,7 +7523,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":5}</t>
+{"evidence":[[610,508,722,620]],"answer":5}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -7537,12 +7537,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 524.0, 714.0, 636.0]], "answer": 20}</t>
+          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 20}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 524.0, 714.0, 636.0]]</t>
+          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -7684,7 +7684,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -7698,12 +7698,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -7748,7 +7748,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -7762,12 +7762,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 16}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 16}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7812,7 +7812,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -7826,12 +7826,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 14}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -7876,7 +7876,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -7890,12 +7890,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -7940,7 +7940,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -7954,12 +7954,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -8004,7 +8004,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -8018,12 +8018,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -8068,7 +8068,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -8082,12 +8082,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 3}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -8132,7 +8132,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -8146,12 +8146,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -8196,7 +8196,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -8210,12 +8210,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -8260,7 +8260,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -8274,12 +8274,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -8324,7 +8324,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -8338,12 +8338,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -8388,7 +8388,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -8402,12 +8402,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 18}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 18}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -8452,7 +8452,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -8466,12 +8466,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -8516,7 +8516,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -8530,12 +8530,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -8580,7 +8580,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -8594,12 +8594,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 16}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 16}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -8644,7 +8644,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -8658,12 +8658,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -8708,7 +8708,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -8722,12 +8722,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -8772,7 +8772,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -8786,12 +8786,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -8836,7 +8836,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -8850,12 +8850,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -8900,7 +8900,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -8914,12 +8914,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -8964,7 +8964,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -8978,12 +8978,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -9028,7 +9028,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -9042,12 +9042,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -9092,7 +9092,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -9106,12 +9106,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -9156,7 +9156,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -9170,12 +9170,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 14}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -9220,7 +9220,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[574,508,686,620]],"answer":8}</t>
+{"evidence":[[610,508,722,620]],"answer":8}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -9234,12 +9234,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[602.0, 449.0, 714.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[602.0, 449.0, 714.0, 561.0]]</t>
+          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">

</xml_diff>

<commit_message>
puzzles: add balance spacing jitter
</commit_message>
<xml_diff>
--- a/task-reviews/puzzles/task_puzzles_arithmetic_balance_value/task_puzzles_arithmetic_balance_value.xlsx
+++ b/task-reviews/puzzles/task_puzzles_arithmetic_balance_value/task_puzzles_arithmetic_balance_value.xlsx
@@ -4290,7 +4290,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -4304,12 +4304,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 11}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 11}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -4354,7 +4354,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -4368,12 +4368,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -4418,7 +4418,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -4432,12 +4432,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -4482,7 +4482,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4496,12 +4496,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -4546,7 +4546,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4560,12 +4560,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 11}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 11}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -4610,7 +4610,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4624,12 +4624,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 3}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -4674,7 +4674,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -4688,12 +4688,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -4738,7 +4738,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4752,12 +4752,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -4802,7 +4802,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -4816,12 +4816,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -4866,7 +4866,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -4880,12 +4880,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4930,7 +4930,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -4944,12 +4944,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -4994,7 +4994,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -5008,12 +5008,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -5058,7 +5058,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -5072,12 +5072,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 3}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -5122,7 +5122,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -5136,12 +5136,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -5186,7 +5186,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -5200,12 +5200,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 9}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -5250,7 +5250,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -5264,12 +5264,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -5314,7 +5314,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -5328,12 +5328,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -5378,7 +5378,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -5392,12 +5392,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -5442,7 +5442,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -5456,12 +5456,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 5}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -5506,7 +5506,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -5520,12 +5520,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 11}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 11}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -5570,7 +5570,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -5584,12 +5584,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -5634,7 +5634,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -5648,12 +5648,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 8}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5698,7 +5698,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -5712,12 +5712,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -5762,7 +5762,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -5776,12 +5776,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 9}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -5826,7 +5826,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":7}</t>
+{"evidence":[[556,449,668,561]],"answer":7}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -5840,12 +5840,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5987,7 +5987,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -6001,12 +6001,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 4}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -6051,7 +6051,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -6065,12 +6065,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -6115,7 +6115,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -6129,12 +6129,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 2}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -6179,7 +6179,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -6243,7 +6243,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -6257,12 +6257,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 9}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -6307,7 +6307,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -6321,12 +6321,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -6371,7 +6371,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 14}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -6435,7 +6435,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -6449,12 +6449,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 6}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -6499,7 +6499,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -6513,12 +6513,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 16}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 16}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -6563,7 +6563,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -6577,12 +6577,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -6627,7 +6627,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -6641,12 +6641,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 12}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -6691,7 +6691,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -6705,12 +6705,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 14}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -6755,7 +6755,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -6769,12 +6769,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 18}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 18}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -6819,7 +6819,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -6833,12 +6833,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -6883,7 +6883,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -6897,12 +6897,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -6947,7 +6947,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -6961,12 +6961,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 8}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -7011,7 +7011,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -7025,12 +7025,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 9}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 9}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -7075,7 +7075,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -7089,12 +7089,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 2}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -7139,7 +7139,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -7153,12 +7153,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 7}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 7}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -7203,7 +7203,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -7217,12 +7217,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 5}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -7267,7 +7267,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -7281,12 +7281,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 12}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -7331,7 +7331,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -7345,12 +7345,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 8}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 8}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -7395,7 +7395,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -7409,12 +7409,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 10}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -7459,7 +7459,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -7473,12 +7473,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 5}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -7523,7 +7523,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":5}</t>
+{"evidence":[[556,524,668,636]],"answer":5}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -7537,12 +7537,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 524.0, 732.0, 636.0]], "answer": 20}</t>
+          <t>{"evidence": [[555.5, 524.0, 667.5, 636.0]], "answer": 20}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 524.0, 732.0, 636.0]]</t>
+          <t>[[555.5, 524.0, 667.5, 636.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -7684,7 +7684,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -7698,12 +7698,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -7748,7 +7748,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -7762,12 +7762,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 16}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 16}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7812,7 +7812,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -7826,12 +7826,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 14}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -7876,7 +7876,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -7890,12 +7890,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -7940,7 +7940,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -7954,12 +7954,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -8004,7 +8004,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -8018,12 +8018,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -8068,7 +8068,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -8082,12 +8082,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 3}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -8132,7 +8132,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -8146,12 +8146,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -8196,7 +8196,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -8210,12 +8210,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -8260,7 +8260,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -8274,12 +8274,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -8324,7 +8324,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -8338,12 +8338,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -8388,7 +8388,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -8402,12 +8402,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 18}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 18}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -8452,7 +8452,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -8466,12 +8466,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -8516,7 +8516,7 @@
 Evidence field: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer field: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -8530,12 +8530,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -8580,7 +8580,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -8594,12 +8594,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 16}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 16}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -8644,7 +8644,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -8658,12 +8658,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 2}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -8708,7 +8708,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -8722,12 +8722,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -8772,7 +8772,7 @@
 Evidence: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -8786,12 +8786,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -8836,7 +8836,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -8850,12 +8850,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -8900,7 +8900,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -8914,12 +8914,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 6}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 6}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -8964,7 +8964,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -8978,12 +8978,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 10}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 10}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -9028,7 +9028,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -9042,12 +9042,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 12}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 12}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -9092,7 +9092,7 @@
 Evidence format: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer requirement: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -9106,12 +9106,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 1}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -9156,7 +9156,7 @@
 Evidence rule: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer rule: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -9170,12 +9170,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 14}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 14}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -9220,7 +9220,7 @@
 Evidence requirement: set "evidence" to an array containing exactly one bounding box [x1, y1, x2, y2] for the question-mark query box.
 Answer format: set "answer" to the exact integer value requested by the puzzle.
 Example JSON:
-{"evidence":[[610,508,722,620]],"answer":8}</t>
+{"evidence":[[556,449,668,561]],"answer":8}</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -9234,12 +9234,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[620.0, 449.0, 732.0, 561.0]], "answer": 4}</t>
+          <t>{"evidence": [[555.5, 449.0, 667.5, 561.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[620.0, 449.0, 732.0, 561.0]]</t>
+          <t>[[555.5, 449.0, 667.5, 561.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">

</xml_diff>